<commit_message>
Update AGR through September 9 and deliveries through September 4
</commit_message>
<xml_diff>
--- a/Clean_deliveries_format_maize.xlsx
+++ b/Clean_deliveries_format_maize.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\grain-data-intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49EF237-9C23-42B4-935C-79440287D738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{607BC50E-6059-4EDC-98C7-AC9DF03015D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-16200" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-270" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2191" uniqueCount="739">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2192" uniqueCount="740">
   <si>
     <t>SAGIS Week nr</t>
   </si>
@@ -2253,6 +2253,9 @@
   </si>
   <si>
     <t>22/08 - 28/08/2026</t>
+  </si>
+  <si>
+    <t>29/08 - 04/09/2026</t>
   </si>
 </sst>
 </file>
@@ -2687,7 +2690,7 @@
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2815,6 +2818,7 @@
     <xf numFmtId="0" fontId="9" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -56425,19 +56429,19 @@
         <v>137597</v>
       </c>
       <c r="J682" s="10">
-        <v>3365</v>
+        <v>3294</v>
       </c>
       <c r="K682" s="10">
-        <v>140962</v>
+        <v>140891</v>
       </c>
       <c r="L682" s="10">
         <v>205271</v>
       </c>
       <c r="M682" s="10">
-        <v>3877</v>
+        <v>3806</v>
       </c>
       <c r="N682" s="10">
-        <v>209148</v>
+        <v>209077</v>
       </c>
       <c r="O682" s="10">
         <v>64145</v>
@@ -56455,7 +56459,7 @@
         <v>68186</v>
       </c>
       <c r="T682" s="10">
-        <v>137961</v>
+        <v>137890</v>
       </c>
       <c r="U682" s="10">
         <v>2859</v>
@@ -56467,10 +56471,10 @@
         <v>37</v>
       </c>
       <c r="X682" s="10">
-        <v>140962</v>
+        <v>140891</v>
       </c>
       <c r="Y682" s="10">
-        <v>209148</v>
+        <v>209077</v>
       </c>
       <c r="AA682" s="57"/>
     </row>
@@ -56581,19 +56585,19 @@
         <v>412859</v>
       </c>
       <c r="J684" s="10">
-        <v>31474</v>
+        <v>31367</v>
       </c>
       <c r="K684" s="10">
-        <v>444333</v>
+        <v>444226</v>
       </c>
       <c r="L684" s="10">
         <v>614274</v>
       </c>
       <c r="M684" s="10">
-        <v>44156</v>
+        <v>44049</v>
       </c>
       <c r="N684" s="10">
-        <v>658430</v>
+        <v>658323</v>
       </c>
       <c r="O684" s="10">
         <v>205162</v>
@@ -56611,7 +56615,7 @@
         <v>214097</v>
       </c>
       <c r="T684" s="10">
-        <v>420583</v>
+        <v>420476</v>
       </c>
       <c r="U684" s="10">
         <v>23148</v>
@@ -56623,10 +56627,10 @@
         <v>47</v>
       </c>
       <c r="X684" s="10">
-        <v>444333</v>
+        <v>444226</v>
       </c>
       <c r="Y684" s="10">
-        <v>658430</v>
+        <v>658323</v>
       </c>
       <c r="AA684" s="57"/>
     </row>
@@ -56724,64 +56728,64 @@
       <c r="E686" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F686" s="6">
+      <c r="F686" s="63">
         <v>517618</v>
       </c>
-      <c r="G686" s="6">
+      <c r="G686" s="63">
         <v>7338</v>
       </c>
-      <c r="H686" s="6">
+      <c r="H686" s="63">
         <v>524956</v>
       </c>
-      <c r="I686" s="6">
+      <c r="I686" s="63">
         <v>592608</v>
       </c>
-      <c r="J686" s="6">
+      <c r="J686" s="63">
         <v>7187</v>
       </c>
-      <c r="K686" s="6">
+      <c r="K686" s="63">
         <v>599795</v>
       </c>
-      <c r="L686" s="6">
+      <c r="L686" s="63">
         <v>1110226</v>
       </c>
-      <c r="M686" s="6">
+      <c r="M686" s="63">
         <v>14525</v>
       </c>
-      <c r="N686" s="6">
+      <c r="N686" s="63">
         <v>1124751</v>
       </c>
-      <c r="O686" s="6">
+      <c r="O686" s="63">
         <v>496961</v>
       </c>
-      <c r="P686" s="6">
+      <c r="P686" s="63">
         <v>26631</v>
       </c>
-      <c r="Q686" s="6">
+      <c r="Q686" s="63">
         <v>1187</v>
       </c>
       <c r="R686" s="6">
         <v>177</v>
       </c>
-      <c r="S686" s="6">
+      <c r="S686" s="63">
         <v>524956</v>
       </c>
-      <c r="T686" s="6">
+      <c r="T686" s="63">
         <v>542083</v>
       </c>
-      <c r="U686" s="6">
+      <c r="U686" s="63">
         <v>54295</v>
       </c>
-      <c r="V686" s="6">
+      <c r="V686" s="63">
         <v>3228</v>
       </c>
       <c r="W686" s="6">
         <v>189</v>
       </c>
-      <c r="X686" s="6">
+      <c r="X686" s="63">
         <v>599795</v>
       </c>
-      <c r="Y686" s="6">
+      <c r="Y686" s="63">
         <v>1124751</v>
       </c>
       <c r="AA686" s="57"/>
@@ -56802,65 +56806,65 @@
       <c r="E687" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F687" s="6">
+      <c r="F687" s="63">
         <v>702695</v>
       </c>
-      <c r="G687" s="6">
+      <c r="G687" s="63">
         <v>8754</v>
       </c>
-      <c r="H687" s="6">
+      <c r="H687" s="63">
         <v>711449</v>
       </c>
-      <c r="I687" s="6">
+      <c r="I687" s="63">
         <v>669414</v>
       </c>
-      <c r="J687" s="6">
-        <v>6344</v>
-      </c>
-      <c r="K687" s="6">
-        <v>675758</v>
-      </c>
-      <c r="L687" s="6">
+      <c r="J687" s="63">
+        <v>6345</v>
+      </c>
+      <c r="K687" s="63">
+        <v>675759</v>
+      </c>
+      <c r="L687" s="63">
         <v>1372109</v>
       </c>
-      <c r="M687" s="6">
-        <v>15098</v>
-      </c>
-      <c r="N687" s="6">
-        <v>1387207</v>
-      </c>
-      <c r="O687" s="6">
+      <c r="M687" s="63">
+        <v>15099</v>
+      </c>
+      <c r="N687" s="63">
+        <v>1387208</v>
+      </c>
+      <c r="O687" s="63">
         <v>674799</v>
       </c>
-      <c r="P687" s="6">
+      <c r="P687" s="63">
         <v>34795</v>
       </c>
-      <c r="Q687" s="6">
+      <c r="Q687" s="63">
         <v>1810</v>
       </c>
       <c r="R687" s="6">
         <v>45</v>
       </c>
-      <c r="S687" s="6">
+      <c r="S687" s="63">
         <v>711449</v>
       </c>
-      <c r="T687" s="6">
-        <v>614475</v>
-      </c>
-      <c r="U687" s="6">
+      <c r="T687" s="63">
+        <v>614476</v>
+      </c>
+      <c r="U687" s="63">
         <v>57879</v>
       </c>
-      <c r="V687" s="6">
+      <c r="V687" s="63">
         <v>3266</v>
       </c>
       <c r="W687" s="6">
         <v>138</v>
       </c>
-      <c r="X687" s="6">
-        <v>675758</v>
-      </c>
-      <c r="Y687" s="6">
-        <v>1387207</v>
+      <c r="X687" s="63">
+        <v>675759</v>
+      </c>
+      <c r="Y687" s="63">
+        <v>1387208</v>
       </c>
     </row>
     <row r="688" spans="1:27" x14ac:dyDescent="0.25">
@@ -56879,52 +56883,52 @@
       <c r="E688" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F688" s="6">
+      <c r="F688" s="63">
         <v>456498</v>
       </c>
-      <c r="G688" s="6">
+      <c r="G688" s="63">
         <v>47110</v>
       </c>
-      <c r="H688" s="6">
+      <c r="H688" s="63">
         <v>503608</v>
       </c>
-      <c r="I688" s="6">
+      <c r="I688" s="63">
         <v>390877</v>
       </c>
-      <c r="J688" s="6">
-        <v>75176</v>
-      </c>
-      <c r="K688" s="6">
-        <v>466053</v>
-      </c>
-      <c r="L688" s="6">
+      <c r="J688" s="63">
+        <v>75213</v>
+      </c>
+      <c r="K688" s="63">
+        <v>466090</v>
+      </c>
+      <c r="L688" s="63">
         <v>847375</v>
       </c>
-      <c r="M688" s="6">
-        <v>122286</v>
-      </c>
-      <c r="N688" s="6">
-        <v>969661</v>
-      </c>
-      <c r="O688" s="6">
+      <c r="M688" s="63">
+        <v>122323</v>
+      </c>
+      <c r="N688" s="63">
+        <v>969698</v>
+      </c>
+      <c r="O688" s="63">
         <v>476358</v>
       </c>
-      <c r="P688" s="6">
+      <c r="P688" s="63">
         <v>24451</v>
       </c>
-      <c r="Q688" s="6">
+      <c r="Q688" s="63">
         <v>2763</v>
       </c>
       <c r="R688" s="6">
         <v>36</v>
       </c>
-      <c r="S688" s="6">
+      <c r="S688" s="63">
         <v>503608</v>
       </c>
-      <c r="T688" s="6">
-        <v>433502</v>
-      </c>
-      <c r="U688" s="6">
+      <c r="T688" s="63">
+        <v>433539</v>
+      </c>
+      <c r="U688" s="63">
         <v>31539</v>
       </c>
       <c r="V688" s="6">
@@ -56933,11 +56937,11 @@
       <c r="W688" s="6">
         <v>188</v>
       </c>
-      <c r="X688" s="6">
-        <v>466053</v>
-      </c>
-      <c r="Y688" s="6">
-        <v>969661</v>
+      <c r="X688" s="63">
+        <v>466090</v>
+      </c>
+      <c r="Y688" s="63">
+        <v>969698</v>
       </c>
     </row>
     <row r="689" spans="1:25" x14ac:dyDescent="0.25">
@@ -56956,64 +56960,64 @@
       <c r="E689" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F689" s="6">
+      <c r="F689" s="63">
         <v>488226</v>
       </c>
-      <c r="G689" s="6">
+      <c r="G689" s="63">
         <v>33395</v>
       </c>
-      <c r="H689" s="6">
+      <c r="H689" s="63">
         <v>521621</v>
       </c>
-      <c r="I689" s="6">
+      <c r="I689" s="63">
         <v>379489</v>
       </c>
-      <c r="J689" s="6">
+      <c r="J689" s="63">
         <v>13568</v>
       </c>
-      <c r="K689" s="6">
+      <c r="K689" s="63">
         <v>393057</v>
       </c>
-      <c r="L689" s="6">
+      <c r="L689" s="63">
         <v>867715</v>
       </c>
-      <c r="M689" s="6">
+      <c r="M689" s="63">
         <v>46963</v>
       </c>
-      <c r="N689" s="6">
+      <c r="N689" s="63">
         <v>914678</v>
       </c>
-      <c r="O689" s="6">
+      <c r="O689" s="63">
         <v>492424</v>
       </c>
-      <c r="P689" s="6">
+      <c r="P689" s="63">
         <v>26156</v>
       </c>
-      <c r="Q689" s="6">
+      <c r="Q689" s="63">
         <v>2991</v>
       </c>
       <c r="R689" s="6">
         <v>50</v>
       </c>
-      <c r="S689" s="6">
+      <c r="S689" s="63">
         <v>521621</v>
       </c>
-      <c r="T689" s="6">
+      <c r="T689" s="63">
         <v>358381</v>
       </c>
-      <c r="U689" s="6">
+      <c r="U689" s="63">
         <v>33163</v>
       </c>
-      <c r="V689" s="6">
+      <c r="V689" s="63">
         <v>1443</v>
       </c>
       <c r="W689" s="6">
         <v>70</v>
       </c>
-      <c r="X689" s="6">
+      <c r="X689" s="63">
         <v>393057</v>
       </c>
-      <c r="Y689" s="6">
+      <c r="Y689" s="63">
         <v>914678</v>
       </c>
     </row>
@@ -57033,65 +57037,65 @@
       <c r="E690" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F690" s="6">
+      <c r="F690" s="63">
         <v>833175</v>
       </c>
-      <c r="G690" s="6">
+      <c r="G690" s="63">
         <v>10521</v>
       </c>
-      <c r="H690" s="6">
+      <c r="H690" s="63">
         <v>843696</v>
       </c>
-      <c r="I690" s="6">
+      <c r="I690" s="63">
         <v>556930</v>
       </c>
-      <c r="J690" s="6">
-        <v>6584</v>
-      </c>
-      <c r="K690" s="6">
-        <v>563514</v>
-      </c>
-      <c r="L690" s="6">
+      <c r="J690" s="63">
+        <v>6585</v>
+      </c>
+      <c r="K690" s="63">
+        <v>563515</v>
+      </c>
+      <c r="L690" s="63">
         <v>1390105</v>
       </c>
-      <c r="M690" s="6">
-        <v>17105</v>
-      </c>
-      <c r="N690" s="6">
-        <v>1407210</v>
-      </c>
-      <c r="O690" s="6">
+      <c r="M690" s="63">
+        <v>17106</v>
+      </c>
+      <c r="N690" s="63">
+        <v>1407211</v>
+      </c>
+      <c r="O690" s="63">
         <v>795990</v>
       </c>
-      <c r="P690" s="6">
+      <c r="P690" s="63">
         <v>42184</v>
       </c>
-      <c r="Q690" s="6">
+      <c r="Q690" s="63">
         <v>5458</v>
       </c>
       <c r="R690" s="6">
         <v>64</v>
       </c>
-      <c r="S690" s="6">
+      <c r="S690" s="63">
         <v>843696</v>
       </c>
-      <c r="T690" s="6">
-        <v>502613</v>
-      </c>
-      <c r="U690" s="6">
+      <c r="T690" s="63">
+        <v>502614</v>
+      </c>
+      <c r="U690" s="63">
         <v>58757</v>
       </c>
-      <c r="V690" s="6">
+      <c r="V690" s="63">
         <v>2013</v>
       </c>
       <c r="W690" s="6">
         <v>131</v>
       </c>
-      <c r="X690" s="6">
-        <v>563514</v>
-      </c>
-      <c r="Y690" s="6">
-        <v>1407210</v>
+      <c r="X690" s="63">
+        <v>563515</v>
+      </c>
+      <c r="Y690" s="63">
+        <v>1407211</v>
       </c>
     </row>
     <row r="691" spans="1:25" x14ac:dyDescent="0.25">
@@ -57110,65 +57114,65 @@
       <c r="E691" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F691" s="6">
+      <c r="F691" s="63">
         <v>915075</v>
       </c>
-      <c r="G691" s="6">
+      <c r="G691" s="63">
         <v>59905</v>
       </c>
-      <c r="H691" s="6">
+      <c r="H691" s="63">
         <v>974980</v>
       </c>
-      <c r="I691" s="6">
+      <c r="I691" s="63">
         <v>550540</v>
       </c>
-      <c r="J691" s="6">
-        <v>43925</v>
-      </c>
-      <c r="K691" s="6">
-        <v>594465</v>
-      </c>
-      <c r="L691" s="6">
+      <c r="J691" s="63">
+        <v>43631</v>
+      </c>
+      <c r="K691" s="63">
+        <v>594171</v>
+      </c>
+      <c r="L691" s="63">
         <v>1465615</v>
       </c>
-      <c r="M691" s="6">
-        <v>103830</v>
-      </c>
-      <c r="N691" s="6">
-        <v>1569445</v>
-      </c>
-      <c r="O691" s="6">
+      <c r="M691" s="63">
+        <v>103536</v>
+      </c>
+      <c r="N691" s="63">
+        <v>1569151</v>
+      </c>
+      <c r="O691" s="63">
         <v>911715</v>
       </c>
-      <c r="P691" s="6">
+      <c r="P691" s="63">
         <v>58498</v>
       </c>
-      <c r="Q691" s="6">
+      <c r="Q691" s="63">
         <v>4689</v>
       </c>
       <c r="R691" s="6">
         <v>78</v>
       </c>
-      <c r="S691" s="6">
+      <c r="S691" s="63">
         <v>974980</v>
       </c>
-      <c r="T691" s="6">
-        <v>530648</v>
-      </c>
-      <c r="U691" s="6">
+      <c r="T691" s="63">
+        <v>530354</v>
+      </c>
+      <c r="U691" s="63">
         <v>60129</v>
       </c>
-      <c r="V691" s="6">
+      <c r="V691" s="63">
         <v>3580</v>
       </c>
       <c r="W691" s="6">
         <v>108</v>
       </c>
-      <c r="X691" s="6">
-        <v>594465</v>
-      </c>
-      <c r="Y691" s="6">
-        <v>1569445</v>
+      <c r="X691" s="63">
+        <v>594171</v>
+      </c>
+      <c r="Y691" s="63">
+        <v>1569151</v>
       </c>
     </row>
     <row r="692" spans="1:25" x14ac:dyDescent="0.25">
@@ -57187,65 +57191,65 @@
       <c r="E692" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F692" s="6">
+      <c r="F692" s="63">
         <v>937765</v>
       </c>
-      <c r="G692" s="6">
+      <c r="G692" s="63">
         <v>12002</v>
       </c>
-      <c r="H692" s="6">
+      <c r="H692" s="63">
         <v>949767</v>
       </c>
-      <c r="I692" s="6">
+      <c r="I692" s="63">
         <v>445313</v>
       </c>
-      <c r="J692" s="6">
-        <v>15527</v>
-      </c>
-      <c r="K692" s="6">
-        <v>460840</v>
-      </c>
-      <c r="L692" s="6">
+      <c r="J692" s="63">
+        <v>15530</v>
+      </c>
+      <c r="K692" s="63">
+        <v>460843</v>
+      </c>
+      <c r="L692" s="63">
         <v>1383078</v>
       </c>
-      <c r="M692" s="6">
-        <v>27529</v>
-      </c>
-      <c r="N692" s="6">
-        <v>1410607</v>
-      </c>
-      <c r="O692" s="6">
+      <c r="M692" s="63">
+        <v>27532</v>
+      </c>
+      <c r="N692" s="63">
+        <v>1410610</v>
+      </c>
+      <c r="O692" s="63">
         <v>885551</v>
       </c>
-      <c r="P692" s="6">
+      <c r="P692" s="63">
         <v>61516</v>
       </c>
-      <c r="Q692" s="6">
+      <c r="Q692" s="63">
         <v>2678</v>
       </c>
       <c r="R692" s="6">
         <v>22</v>
       </c>
-      <c r="S692" s="6">
+      <c r="S692" s="63">
         <v>949767</v>
       </c>
-      <c r="T692" s="6">
-        <v>405590</v>
-      </c>
-      <c r="U692" s="6">
+      <c r="T692" s="63">
+        <v>405593</v>
+      </c>
+      <c r="U692" s="63">
         <v>52483</v>
       </c>
-      <c r="V692" s="6">
+      <c r="V692" s="63">
         <v>2697</v>
       </c>
       <c r="W692" s="6">
         <v>70</v>
       </c>
-      <c r="X692" s="6">
-        <v>460840</v>
-      </c>
-      <c r="Y692" s="6">
-        <v>1410607</v>
+      <c r="X692" s="63">
+        <v>460843</v>
+      </c>
+      <c r="Y692" s="63">
+        <v>1410610</v>
       </c>
     </row>
     <row r="693" spans="1:25" x14ac:dyDescent="0.25">
@@ -57264,52 +57268,52 @@
       <c r="E693" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F693" s="6">
+      <c r="F693" s="63">
         <v>800679</v>
       </c>
-      <c r="G693" s="6">
+      <c r="G693" s="63">
         <v>51711</v>
       </c>
-      <c r="H693" s="6">
+      <c r="H693" s="63">
         <v>852390</v>
       </c>
-      <c r="I693" s="6">
+      <c r="I693" s="63">
         <v>343793</v>
       </c>
-      <c r="J693" s="6">
-        <v>76033</v>
-      </c>
-      <c r="K693" s="6">
-        <v>419826</v>
-      </c>
-      <c r="L693" s="6">
+      <c r="J693" s="63">
+        <v>75766</v>
+      </c>
+      <c r="K693" s="63">
+        <v>419559</v>
+      </c>
+      <c r="L693" s="63">
         <v>1144472</v>
       </c>
-      <c r="M693" s="6">
-        <v>127744</v>
-      </c>
-      <c r="N693" s="6">
-        <v>1272216</v>
-      </c>
-      <c r="O693" s="6">
+      <c r="M693" s="63">
+        <v>127477</v>
+      </c>
+      <c r="N693" s="63">
+        <v>1271949</v>
+      </c>
+      <c r="O693" s="63">
         <v>786453</v>
       </c>
-      <c r="P693" s="6">
+      <c r="P693" s="63">
         <v>62303</v>
       </c>
-      <c r="Q693" s="6">
+      <c r="Q693" s="63">
         <v>3628</v>
       </c>
       <c r="R693" s="6">
         <v>6</v>
       </c>
-      <c r="S693" s="6">
+      <c r="S693" s="63">
         <v>852390</v>
       </c>
-      <c r="T693" s="6">
-        <v>378233</v>
-      </c>
-      <c r="U693" s="6">
+      <c r="T693" s="63">
+        <v>377966</v>
+      </c>
+      <c r="U693" s="63">
         <v>40682</v>
       </c>
       <c r="V693" s="6">
@@ -57318,11 +57322,11 @@
       <c r="W693" s="6">
         <v>24</v>
       </c>
-      <c r="X693" s="6">
-        <v>419826</v>
-      </c>
-      <c r="Y693" s="6">
-        <v>1272216</v>
+      <c r="X693" s="63">
+        <v>419559</v>
+      </c>
+      <c r="Y693" s="63">
+        <v>1271949</v>
       </c>
     </row>
     <row r="694" spans="1:25" x14ac:dyDescent="0.25">
@@ -57341,52 +57345,52 @@
       <c r="E694" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F694" s="6">
+      <c r="F694" s="63">
         <v>637394</v>
       </c>
-      <c r="G694" s="6">
-        <v>1241</v>
-      </c>
-      <c r="H694" s="6">
-        <v>638635</v>
-      </c>
-      <c r="I694" s="6">
+      <c r="G694" s="63">
+        <v>1169</v>
+      </c>
+      <c r="H694" s="63">
+        <v>638563</v>
+      </c>
+      <c r="I694" s="63">
         <v>257890</v>
       </c>
-      <c r="J694" s="6">
+      <c r="J694" s="63">
         <v>1542</v>
       </c>
-      <c r="K694" s="6">
+      <c r="K694" s="63">
         <v>259432</v>
       </c>
-      <c r="L694" s="6">
+      <c r="L694" s="63">
         <v>895284</v>
       </c>
-      <c r="M694" s="6">
-        <v>2783</v>
-      </c>
-      <c r="N694" s="6">
-        <v>898067</v>
-      </c>
-      <c r="O694" s="6">
-        <v>573907</v>
-      </c>
-      <c r="P694" s="6">
+      <c r="M694" s="63">
+        <v>2711</v>
+      </c>
+      <c r="N694" s="63">
+        <v>897995</v>
+      </c>
+      <c r="O694" s="63">
+        <v>573835</v>
+      </c>
+      <c r="P694" s="63">
         <v>61784</v>
       </c>
-      <c r="Q694" s="6">
+      <c r="Q694" s="63">
         <v>2918</v>
       </c>
       <c r="R694" s="6">
         <v>26</v>
       </c>
-      <c r="S694" s="6">
-        <v>638635</v>
-      </c>
-      <c r="T694" s="6">
+      <c r="S694" s="63">
+        <v>638563</v>
+      </c>
+      <c r="T694" s="63">
         <v>230287</v>
       </c>
-      <c r="U694" s="6">
+      <c r="U694" s="63">
         <v>28327</v>
       </c>
       <c r="V694" s="6">
@@ -57395,11 +57399,11 @@
       <c r="W694" s="6">
         <v>35</v>
       </c>
-      <c r="X694" s="6">
+      <c r="X694" s="63">
         <v>259432</v>
       </c>
-      <c r="Y694" s="6">
-        <v>898067</v>
+      <c r="Y694" s="63">
+        <v>897995</v>
       </c>
     </row>
     <row r="695" spans="1:25" x14ac:dyDescent="0.25">
@@ -57418,52 +57422,52 @@
       <c r="E695" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F695" s="6">
+      <c r="F695" s="63">
         <v>268544</v>
       </c>
       <c r="G695" s="6">
         <v>991</v>
       </c>
-      <c r="H695" s="6">
+      <c r="H695" s="63">
         <v>269535</v>
       </c>
-      <c r="I695" s="6">
+      <c r="I695" s="63">
         <v>85485</v>
       </c>
-      <c r="J695" s="6">
+      <c r="J695" s="63">
         <v>2628</v>
       </c>
-      <c r="K695" s="6">
+      <c r="K695" s="63">
         <v>88113</v>
       </c>
-      <c r="L695" s="6">
+      <c r="L695" s="63">
         <v>354029</v>
       </c>
-      <c r="M695" s="6">
+      <c r="M695" s="63">
         <v>3619</v>
       </c>
-      <c r="N695" s="6">
+      <c r="N695" s="63">
         <v>357648</v>
       </c>
-      <c r="O695" s="6">
+      <c r="O695" s="63">
         <v>237522</v>
       </c>
-      <c r="P695" s="6">
+      <c r="P695" s="63">
         <v>30086</v>
       </c>
-      <c r="Q695" s="6">
+      <c r="Q695" s="63">
         <v>1923</v>
       </c>
       <c r="R695" s="6">
         <v>4</v>
       </c>
-      <c r="S695" s="6">
+      <c r="S695" s="63">
         <v>269535</v>
       </c>
-      <c r="T695" s="6">
+      <c r="T695" s="63">
         <v>80880</v>
       </c>
-      <c r="U695" s="6">
+      <c r="U695" s="63">
         <v>6843</v>
       </c>
       <c r="V695" s="6">
@@ -57472,10 +57476,10 @@
       <c r="W695" s="6">
         <v>304</v>
       </c>
-      <c r="X695" s="6">
+      <c r="X695" s="63">
         <v>88113</v>
       </c>
-      <c r="Y695" s="6">
+      <c r="Y695" s="63">
         <v>357648</v>
       </c>
     </row>
@@ -57495,52 +57499,52 @@
       <c r="E696" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F696" s="6">
+      <c r="F696" s="63">
         <v>432804</v>
       </c>
-      <c r="G696" s="6">
+      <c r="G696" s="63">
         <v>-5334</v>
       </c>
-      <c r="H696" s="6">
+      <c r="H696" s="63">
         <v>427470</v>
       </c>
-      <c r="I696" s="6">
+      <c r="I696" s="63">
         <v>150038</v>
       </c>
       <c r="J696" s="6">
-        <v>1140</v>
-      </c>
-      <c r="K696" s="6">
-        <v>151178</v>
-      </c>
-      <c r="L696" s="6">
+        <v>956</v>
+      </c>
+      <c r="K696" s="63">
+        <v>150994</v>
+      </c>
+      <c r="L696" s="63">
         <v>582842</v>
       </c>
-      <c r="M696" s="6">
-        <v>-4194</v>
-      </c>
-      <c r="N696" s="6">
-        <v>578648</v>
-      </c>
-      <c r="O696" s="6">
+      <c r="M696" s="63">
+        <v>-4378</v>
+      </c>
+      <c r="N696" s="63">
+        <v>578464</v>
+      </c>
+      <c r="O696" s="63">
         <v>374492</v>
       </c>
-      <c r="P696" s="6">
+      <c r="P696" s="63">
         <v>48627</v>
       </c>
-      <c r="Q696" s="6">
+      <c r="Q696" s="63">
         <v>4323</v>
       </c>
       <c r="R696" s="6">
         <v>28</v>
       </c>
-      <c r="S696" s="6">
+      <c r="S696" s="63">
         <v>427470</v>
       </c>
-      <c r="T696" s="6">
-        <v>135290</v>
-      </c>
-      <c r="U696" s="6">
+      <c r="T696" s="63">
+        <v>135106</v>
+      </c>
+      <c r="U696" s="63">
         <v>15007</v>
       </c>
       <c r="V696" s="6">
@@ -57549,11 +57553,11 @@
       <c r="W696" s="6">
         <v>7</v>
       </c>
-      <c r="X696" s="6">
-        <v>151178</v>
-      </c>
-      <c r="Y696" s="6">
-        <v>578648</v>
+      <c r="X696" s="63">
+        <v>150994</v>
+      </c>
+      <c r="Y696" s="63">
+        <v>578464</v>
       </c>
     </row>
     <row r="697" spans="1:25" x14ac:dyDescent="0.25">
@@ -57572,52 +57576,52 @@
       <c r="E697" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F697" s="6">
+      <c r="F697" s="63">
         <v>260568</v>
       </c>
-      <c r="G697" s="6">
-        <v>0</v>
-      </c>
-      <c r="H697" s="6">
-        <v>260568</v>
-      </c>
-      <c r="I697" s="6">
+      <c r="G697" s="63">
+        <v>4183</v>
+      </c>
+      <c r="H697" s="63">
+        <v>264751</v>
+      </c>
+      <c r="I697" s="63">
         <v>109681</v>
       </c>
-      <c r="J697" s="6">
-        <v>0</v>
-      </c>
-      <c r="K697" s="6">
-        <v>109681</v>
-      </c>
-      <c r="L697" s="6">
+      <c r="J697" s="63">
+        <v>8812</v>
+      </c>
+      <c r="K697" s="63">
+        <v>118493</v>
+      </c>
+      <c r="L697" s="63">
         <v>370249</v>
       </c>
-      <c r="M697" s="6">
-        <v>0</v>
-      </c>
-      <c r="N697" s="6">
-        <v>370249</v>
-      </c>
-      <c r="O697" s="6">
-        <v>230737</v>
-      </c>
-      <c r="P697" s="6">
+      <c r="M697" s="63">
+        <v>12995</v>
+      </c>
+      <c r="N697" s="63">
+        <v>383244</v>
+      </c>
+      <c r="O697" s="63">
+        <v>234920</v>
+      </c>
+      <c r="P697" s="63">
         <v>26757</v>
       </c>
-      <c r="Q697" s="6">
+      <c r="Q697" s="63">
         <v>3065</v>
       </c>
       <c r="R697" s="6">
         <v>9</v>
       </c>
-      <c r="S697" s="6">
-        <v>260568</v>
-      </c>
-      <c r="T697" s="6">
-        <v>101143</v>
-      </c>
-      <c r="U697" s="6">
+      <c r="S697" s="63">
+        <v>264751</v>
+      </c>
+      <c r="T697" s="63">
+        <v>109955</v>
+      </c>
+      <c r="U697" s="63">
         <v>8174</v>
       </c>
       <c r="V697" s="6">
@@ -57626,11 +57630,11 @@
       <c r="W697" s="6">
         <v>60</v>
       </c>
-      <c r="X697" s="6">
-        <v>109681</v>
-      </c>
-      <c r="Y697" s="6">
-        <v>370249</v>
+      <c r="X697" s="63">
+        <v>118493</v>
+      </c>
+      <c r="Y697" s="63">
+        <v>383244</v>
       </c>
     </row>
     <row r="698" spans="1:25" x14ac:dyDescent="0.25">
@@ -57640,33 +57644,75 @@
       <c r="B698" s="4">
         <v>27</v>
       </c>
-      <c r="C698" s="7"/>
+      <c r="C698" s="60" t="s">
+        <v>739</v>
+      </c>
       <c r="D698" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E698" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F698" s="6"/>
-      <c r="G698" s="6"/>
-      <c r="H698" s="6"/>
-      <c r="I698" s="6"/>
-      <c r="J698" s="6"/>
-      <c r="K698" s="6"/>
-      <c r="L698" s="6"/>
-      <c r="M698" s="6"/>
-      <c r="N698" s="6"/>
-      <c r="O698" s="6"/>
-      <c r="P698" s="6"/>
-      <c r="Q698" s="6"/>
-      <c r="R698" s="6"/>
-      <c r="S698" s="6"/>
-      <c r="T698" s="6"/>
-      <c r="U698" s="6"/>
-      <c r="V698" s="6"/>
-      <c r="W698" s="6"/>
-      <c r="X698" s="6"/>
-      <c r="Y698" s="6"/>
+      <c r="F698" s="63">
+        <v>146617</v>
+      </c>
+      <c r="G698" s="6">
+        <v>0</v>
+      </c>
+      <c r="H698" s="63">
+        <v>146617</v>
+      </c>
+      <c r="I698" s="63">
+        <v>77228</v>
+      </c>
+      <c r="J698" s="6">
+        <v>0</v>
+      </c>
+      <c r="K698" s="63">
+        <v>77228</v>
+      </c>
+      <c r="L698" s="63">
+        <v>223845</v>
+      </c>
+      <c r="M698" s="6">
+        <v>0</v>
+      </c>
+      <c r="N698" s="63">
+        <v>223845</v>
+      </c>
+      <c r="O698" s="63">
+        <v>130250</v>
+      </c>
+      <c r="P698" s="63">
+        <v>14724</v>
+      </c>
+      <c r="Q698" s="63">
+        <v>1588</v>
+      </c>
+      <c r="R698" s="6">
+        <v>55</v>
+      </c>
+      <c r="S698" s="63">
+        <v>146617</v>
+      </c>
+      <c r="T698" s="63">
+        <v>71292</v>
+      </c>
+      <c r="U698" s="63">
+        <v>5916</v>
+      </c>
+      <c r="V698" s="6">
+        <v>20</v>
+      </c>
+      <c r="W698" s="6">
+        <v>0</v>
+      </c>
+      <c r="X698" s="63">
+        <v>77228</v>
+      </c>
+      <c r="Y698" s="63">
+        <v>223845</v>
+      </c>
     </row>
     <row r="699" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A699" s="7">
@@ -58813,6 +58859,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075ECE796D7EABA42BC0DB2CA73C7CE00" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e2ecee1b3d34a959aed38d5dc4c878f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8" xmlns:ns3="ae149517-eeaa-465d-b3b6-396a1e23bc6e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9af26d9f7c79c0f2a842447557dfee25" ns2:_="" ns3:_="">
     <xsd:import namespace="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
@@ -59039,17 +59096,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -59060,6 +59106,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
+    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A42C790-3343-4FC1-9ABA-46A7C5CDBF94}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -59078,17 +59135,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
-    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update deliveries through October 9 and wheat 2026/27 estimate
</commit_message>
<xml_diff>
--- a/Clean_deliveries_format_maize.xlsx
+++ b/Clean_deliveries_format_maize.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\grain-data-intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{607BC50E-6059-4EDC-98C7-AC9DF03015D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D9FCC37-8CFB-462C-B2CA-5483F186004D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-270" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2192" uniqueCount="740">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2197" uniqueCount="745">
   <si>
     <t>SAGIS Week nr</t>
   </si>
@@ -2256,6 +2256,21 @@
   </si>
   <si>
     <t>29/08 - 04/09/2026</t>
+  </si>
+  <si>
+    <t>05/09 - 11/09/2026</t>
+  </si>
+  <si>
+    <t>12/09 - 18/09/2026</t>
+  </si>
+  <si>
+    <t>19/09 - 25/09/2026</t>
+  </si>
+  <si>
+    <t>26/09 - 02/10/2026</t>
+  </si>
+  <si>
+    <t>03/10 - 09/10/2026</t>
   </si>
 </sst>
 </file>
@@ -2812,13 +2827,13 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3192,11 +3207,11 @@
         <v>76</v>
       </c>
       <c r="AC1" s="45"/>
-      <c r="AD1" s="61" t="s">
+      <c r="AD1" s="62" t="s">
         <v>723</v>
       </c>
-      <c r="AE1" s="61"/>
-      <c r="AF1" s="62"/>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="63"/>
     </row>
     <row r="2" spans="1:32" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="31">
@@ -56342,31 +56357,31 @@
         <v>28999</v>
       </c>
       <c r="G681" s="10">
-        <v>1559</v>
+        <v>112</v>
       </c>
       <c r="H681" s="10">
-        <v>30558</v>
+        <v>29111</v>
       </c>
       <c r="I681" s="10">
         <v>73014</v>
       </c>
       <c r="J681" s="10">
-        <v>385</v>
+        <v>748</v>
       </c>
       <c r="K681" s="10">
-        <v>73399</v>
+        <v>73762</v>
       </c>
       <c r="L681" s="10">
         <v>102013</v>
       </c>
       <c r="M681" s="10">
-        <v>1944</v>
+        <v>860</v>
       </c>
       <c r="N681" s="10">
-        <v>103957</v>
+        <v>102873</v>
       </c>
       <c r="O681" s="10">
-        <v>28645</v>
+        <v>27198</v>
       </c>
       <c r="P681" s="10">
         <v>1766</v>
@@ -56378,10 +56393,10 @@
         <v>91</v>
       </c>
       <c r="S681" s="10">
-        <v>30558</v>
+        <v>29111</v>
       </c>
       <c r="T681" s="10">
-        <v>72084</v>
+        <v>72447</v>
       </c>
       <c r="U681" s="10">
         <v>1182</v>
@@ -56393,10 +56408,10 @@
         <v>78</v>
       </c>
       <c r="X681" s="10">
-        <v>73399</v>
+        <v>73762</v>
       </c>
       <c r="Y681" s="10">
-        <v>103957</v>
+        <v>102873</v>
       </c>
       <c r="AA681" s="57"/>
     </row>
@@ -56420,31 +56435,31 @@
         <v>67674</v>
       </c>
       <c r="G682" s="10">
-        <v>512</v>
+        <v>-758</v>
       </c>
       <c r="H682" s="10">
-        <v>68186</v>
+        <v>66916</v>
       </c>
       <c r="I682" s="10">
         <v>137597</v>
       </c>
       <c r="J682" s="10">
-        <v>3294</v>
+        <v>3510</v>
       </c>
       <c r="K682" s="10">
-        <v>140891</v>
+        <v>141107</v>
       </c>
       <c r="L682" s="10">
         <v>205271</v>
       </c>
       <c r="M682" s="10">
-        <v>3806</v>
+        <v>2752</v>
       </c>
       <c r="N682" s="10">
-        <v>209077</v>
+        <v>208023</v>
       </c>
       <c r="O682" s="10">
-        <v>64145</v>
+        <v>62875</v>
       </c>
       <c r="P682" s="10">
         <v>3968</v>
@@ -56456,10 +56471,10 @@
         <v>38</v>
       </c>
       <c r="S682" s="10">
-        <v>68186</v>
+        <v>66916</v>
       </c>
       <c r="T682" s="10">
-        <v>137890</v>
+        <v>138106</v>
       </c>
       <c r="U682" s="10">
         <v>2859</v>
@@ -56471,10 +56486,10 @@
         <v>37</v>
       </c>
       <c r="X682" s="10">
-        <v>140891</v>
+        <v>141107</v>
       </c>
       <c r="Y682" s="10">
-        <v>209077</v>
+        <v>208023</v>
       </c>
       <c r="AA682" s="57"/>
     </row>
@@ -56498,31 +56513,31 @@
         <v>120859</v>
       </c>
       <c r="G683" s="10">
-        <v>803</v>
+        <v>-461</v>
       </c>
       <c r="H683" s="10">
-        <v>121662</v>
+        <v>120398</v>
       </c>
       <c r="I683" s="10">
         <v>285962</v>
       </c>
       <c r="J683" s="10">
-        <v>3688</v>
+        <v>3758</v>
       </c>
       <c r="K683" s="10">
-        <v>289650</v>
+        <v>289720</v>
       </c>
       <c r="L683" s="10">
         <v>406821</v>
       </c>
       <c r="M683" s="10">
-        <v>4491</v>
+        <v>3297</v>
       </c>
       <c r="N683" s="10">
-        <v>411312</v>
+        <v>410118</v>
       </c>
       <c r="O683" s="10">
-        <v>116369</v>
+        <v>115105</v>
       </c>
       <c r="P683" s="10">
         <v>4462</v>
@@ -56534,10 +56549,10 @@
         <v>111</v>
       </c>
       <c r="S683" s="10">
-        <v>121662</v>
+        <v>120398</v>
       </c>
       <c r="T683" s="10">
-        <v>278292</v>
+        <v>278362</v>
       </c>
       <c r="U683" s="10">
         <v>10777</v>
@@ -56549,10 +56564,10 @@
         <v>2</v>
       </c>
       <c r="X683" s="10">
-        <v>289650</v>
+        <v>289720</v>
       </c>
       <c r="Y683" s="10">
-        <v>411312</v>
+        <v>410118</v>
       </c>
       <c r="AA683" s="57"/>
     </row>
@@ -56576,31 +56591,31 @@
         <v>201415</v>
       </c>
       <c r="G684" s="10">
-        <v>12682</v>
+        <v>16842</v>
       </c>
       <c r="H684" s="10">
-        <v>214097</v>
+        <v>218257</v>
       </c>
       <c r="I684" s="10">
         <v>412859</v>
       </c>
       <c r="J684" s="10">
-        <v>31367</v>
+        <v>31467</v>
       </c>
       <c r="K684" s="10">
-        <v>444226</v>
+        <v>444326</v>
       </c>
       <c r="L684" s="10">
         <v>614274</v>
       </c>
       <c r="M684" s="10">
-        <v>44049</v>
+        <v>48309</v>
       </c>
       <c r="N684" s="10">
-        <v>658323</v>
+        <v>662583</v>
       </c>
       <c r="O684" s="10">
-        <v>205162</v>
+        <v>209322</v>
       </c>
       <c r="P684" s="10">
         <v>8039</v>
@@ -56612,10 +56627,10 @@
         <v>135</v>
       </c>
       <c r="S684" s="10">
-        <v>214097</v>
+        <v>218257</v>
       </c>
       <c r="T684" s="10">
-        <v>420476</v>
+        <v>420576</v>
       </c>
       <c r="U684" s="10">
         <v>23148</v>
@@ -56627,10 +56642,10 @@
         <v>47</v>
       </c>
       <c r="X684" s="10">
-        <v>444226</v>
+        <v>444326</v>
       </c>
       <c r="Y684" s="10">
-        <v>658323</v>
+        <v>662583</v>
       </c>
       <c r="AA684" s="57"/>
     </row>
@@ -56728,64 +56743,64 @@
       <c r="E686" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F686" s="63">
+      <c r="F686" s="61">
         <v>517618</v>
       </c>
-      <c r="G686" s="63">
+      <c r="G686" s="61">
         <v>7338</v>
       </c>
-      <c r="H686" s="63">
+      <c r="H686" s="61">
         <v>524956</v>
       </c>
-      <c r="I686" s="63">
+      <c r="I686" s="61">
         <v>592608</v>
       </c>
-      <c r="J686" s="63">
+      <c r="J686" s="61">
         <v>7187</v>
       </c>
-      <c r="K686" s="63">
+      <c r="K686" s="61">
         <v>599795</v>
       </c>
-      <c r="L686" s="63">
+      <c r="L686" s="61">
         <v>1110226</v>
       </c>
-      <c r="M686" s="63">
+      <c r="M686" s="61">
         <v>14525</v>
       </c>
-      <c r="N686" s="63">
+      <c r="N686" s="61">
         <v>1124751</v>
       </c>
-      <c r="O686" s="63">
+      <c r="O686" s="61">
         <v>496961</v>
       </c>
-      <c r="P686" s="63">
+      <c r="P686" s="61">
         <v>26631</v>
       </c>
-      <c r="Q686" s="63">
+      <c r="Q686" s="61">
         <v>1187</v>
       </c>
       <c r="R686" s="6">
         <v>177</v>
       </c>
-      <c r="S686" s="63">
+      <c r="S686" s="61">
         <v>524956</v>
       </c>
-      <c r="T686" s="63">
+      <c r="T686" s="61">
         <v>542083</v>
       </c>
-      <c r="U686" s="63">
+      <c r="U686" s="61">
         <v>54295</v>
       </c>
-      <c r="V686" s="63">
+      <c r="V686" s="61">
         <v>3228</v>
       </c>
       <c r="W686" s="6">
         <v>189</v>
       </c>
-      <c r="X686" s="63">
+      <c r="X686" s="61">
         <v>599795</v>
       </c>
-      <c r="Y686" s="63">
+      <c r="Y686" s="61">
         <v>1124751</v>
       </c>
       <c r="AA686" s="57"/>
@@ -56806,64 +56821,64 @@
       <c r="E687" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F687" s="63">
+      <c r="F687" s="61">
         <v>702695</v>
       </c>
-      <c r="G687" s="63">
+      <c r="G687" s="61">
         <v>8754</v>
       </c>
-      <c r="H687" s="63">
+      <c r="H687" s="61">
         <v>711449</v>
       </c>
-      <c r="I687" s="63">
+      <c r="I687" s="61">
         <v>669414</v>
       </c>
-      <c r="J687" s="63">
+      <c r="J687" s="61">
         <v>6345</v>
       </c>
-      <c r="K687" s="63">
+      <c r="K687" s="61">
         <v>675759</v>
       </c>
-      <c r="L687" s="63">
+      <c r="L687" s="61">
         <v>1372109</v>
       </c>
-      <c r="M687" s="63">
+      <c r="M687" s="61">
         <v>15099</v>
       </c>
-      <c r="N687" s="63">
+      <c r="N687" s="61">
         <v>1387208</v>
       </c>
-      <c r="O687" s="63">
+      <c r="O687" s="61">
         <v>674799</v>
       </c>
-      <c r="P687" s="63">
+      <c r="P687" s="61">
         <v>34795</v>
       </c>
-      <c r="Q687" s="63">
+      <c r="Q687" s="61">
         <v>1810</v>
       </c>
       <c r="R687" s="6">
         <v>45</v>
       </c>
-      <c r="S687" s="63">
+      <c r="S687" s="61">
         <v>711449</v>
       </c>
-      <c r="T687" s="63">
+      <c r="T687" s="61">
         <v>614476</v>
       </c>
-      <c r="U687" s="63">
+      <c r="U687" s="61">
         <v>57879</v>
       </c>
-      <c r="V687" s="63">
+      <c r="V687" s="61">
         <v>3266</v>
       </c>
       <c r="W687" s="6">
         <v>138</v>
       </c>
-      <c r="X687" s="63">
+      <c r="X687" s="61">
         <v>675759</v>
       </c>
-      <c r="Y687" s="63">
+      <c r="Y687" s="61">
         <v>1387208</v>
       </c>
     </row>
@@ -56883,52 +56898,52 @@
       <c r="E688" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F688" s="63">
+      <c r="F688" s="61">
         <v>456498</v>
       </c>
-      <c r="G688" s="63">
+      <c r="G688" s="61">
         <v>47110</v>
       </c>
-      <c r="H688" s="63">
+      <c r="H688" s="61">
         <v>503608</v>
       </c>
-      <c r="I688" s="63">
+      <c r="I688" s="61">
         <v>390877</v>
       </c>
-      <c r="J688" s="63">
-        <v>75213</v>
-      </c>
-      <c r="K688" s="63">
-        <v>466090</v>
-      </c>
-      <c r="L688" s="63">
+      <c r="J688" s="61">
+        <v>75191</v>
+      </c>
+      <c r="K688" s="61">
+        <v>466068</v>
+      </c>
+      <c r="L688" s="61">
         <v>847375</v>
       </c>
-      <c r="M688" s="63">
-        <v>122323</v>
-      </c>
-      <c r="N688" s="63">
-        <v>969698</v>
-      </c>
-      <c r="O688" s="63">
+      <c r="M688" s="61">
+        <v>122301</v>
+      </c>
+      <c r="N688" s="61">
+        <v>969676</v>
+      </c>
+      <c r="O688" s="61">
         <v>476358</v>
       </c>
-      <c r="P688" s="63">
+      <c r="P688" s="61">
         <v>24451</v>
       </c>
-      <c r="Q688" s="63">
+      <c r="Q688" s="61">
         <v>2763</v>
       </c>
       <c r="R688" s="6">
         <v>36</v>
       </c>
-      <c r="S688" s="63">
+      <c r="S688" s="61">
         <v>503608</v>
       </c>
-      <c r="T688" s="63">
-        <v>433539</v>
-      </c>
-      <c r="U688" s="63">
+      <c r="T688" s="61">
+        <v>433517</v>
+      </c>
+      <c r="U688" s="61">
         <v>31539</v>
       </c>
       <c r="V688" s="6">
@@ -56937,11 +56952,11 @@
       <c r="W688" s="6">
         <v>188</v>
       </c>
-      <c r="X688" s="63">
-        <v>466090</v>
-      </c>
-      <c r="Y688" s="63">
-        <v>969698</v>
+      <c r="X688" s="61">
+        <v>466068</v>
+      </c>
+      <c r="Y688" s="61">
+        <v>969676</v>
       </c>
     </row>
     <row r="689" spans="1:25" x14ac:dyDescent="0.25">
@@ -56960,64 +56975,64 @@
       <c r="E689" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F689" s="63">
+      <c r="F689" s="61">
         <v>488226</v>
       </c>
-      <c r="G689" s="63">
+      <c r="G689" s="61">
         <v>33395</v>
       </c>
-      <c r="H689" s="63">
+      <c r="H689" s="61">
         <v>521621</v>
       </c>
-      <c r="I689" s="63">
+      <c r="I689" s="61">
         <v>379489</v>
       </c>
-      <c r="J689" s="63">
+      <c r="J689" s="61">
         <v>13568</v>
       </c>
-      <c r="K689" s="63">
+      <c r="K689" s="61">
         <v>393057</v>
       </c>
-      <c r="L689" s="63">
+      <c r="L689" s="61">
         <v>867715</v>
       </c>
-      <c r="M689" s="63">
+      <c r="M689" s="61">
         <v>46963</v>
       </c>
-      <c r="N689" s="63">
+      <c r="N689" s="61">
         <v>914678</v>
       </c>
-      <c r="O689" s="63">
+      <c r="O689" s="61">
         <v>492424</v>
       </c>
-      <c r="P689" s="63">
+      <c r="P689" s="61">
         <v>26156</v>
       </c>
-      <c r="Q689" s="63">
+      <c r="Q689" s="61">
         <v>2991</v>
       </c>
       <c r="R689" s="6">
         <v>50</v>
       </c>
-      <c r="S689" s="63">
+      <c r="S689" s="61">
         <v>521621</v>
       </c>
-      <c r="T689" s="63">
+      <c r="T689" s="61">
         <v>358381</v>
       </c>
-      <c r="U689" s="63">
+      <c r="U689" s="61">
         <v>33163</v>
       </c>
-      <c r="V689" s="63">
+      <c r="V689" s="61">
         <v>1443</v>
       </c>
       <c r="W689" s="6">
         <v>70</v>
       </c>
-      <c r="X689" s="63">
+      <c r="X689" s="61">
         <v>393057</v>
       </c>
-      <c r="Y689" s="63">
+      <c r="Y689" s="61">
         <v>914678</v>
       </c>
     </row>
@@ -57037,65 +57052,65 @@
       <c r="E690" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F690" s="63">
+      <c r="F690" s="61">
         <v>833175</v>
       </c>
-      <c r="G690" s="63">
-        <v>10521</v>
-      </c>
-      <c r="H690" s="63">
-        <v>843696</v>
-      </c>
-      <c r="I690" s="63">
+      <c r="G690" s="61">
+        <v>10697</v>
+      </c>
+      <c r="H690" s="61">
+        <v>843872</v>
+      </c>
+      <c r="I690" s="61">
         <v>556930</v>
       </c>
-      <c r="J690" s="63">
+      <c r="J690" s="61">
         <v>6585</v>
       </c>
-      <c r="K690" s="63">
+      <c r="K690" s="61">
         <v>563515</v>
       </c>
-      <c r="L690" s="63">
+      <c r="L690" s="61">
         <v>1390105</v>
       </c>
-      <c r="M690" s="63">
-        <v>17106</v>
-      </c>
-      <c r="N690" s="63">
-        <v>1407211</v>
-      </c>
-      <c r="O690" s="63">
-        <v>795990</v>
-      </c>
-      <c r="P690" s="63">
+      <c r="M690" s="61">
+        <v>17282</v>
+      </c>
+      <c r="N690" s="61">
+        <v>1407387</v>
+      </c>
+      <c r="O690" s="61">
+        <v>796166</v>
+      </c>
+      <c r="P690" s="61">
         <v>42184</v>
       </c>
-      <c r="Q690" s="63">
+      <c r="Q690" s="61">
         <v>5458</v>
       </c>
       <c r="R690" s="6">
         <v>64</v>
       </c>
-      <c r="S690" s="63">
-        <v>843696</v>
-      </c>
-      <c r="T690" s="63">
+      <c r="S690" s="61">
+        <v>843872</v>
+      </c>
+      <c r="T690" s="61">
         <v>502614</v>
       </c>
-      <c r="U690" s="63">
+      <c r="U690" s="61">
         <v>58757</v>
       </c>
-      <c r="V690" s="63">
+      <c r="V690" s="61">
         <v>2013</v>
       </c>
       <c r="W690" s="6">
         <v>131</v>
       </c>
-      <c r="X690" s="63">
+      <c r="X690" s="61">
         <v>563515</v>
       </c>
-      <c r="Y690" s="63">
-        <v>1407211</v>
+      <c r="Y690" s="61">
+        <v>1407387</v>
       </c>
     </row>
     <row r="691" spans="1:25" x14ac:dyDescent="0.25">
@@ -57114,65 +57129,65 @@
       <c r="E691" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F691" s="63">
+      <c r="F691" s="61">
         <v>915075</v>
       </c>
-      <c r="G691" s="63">
-        <v>59905</v>
-      </c>
-      <c r="H691" s="63">
-        <v>974980</v>
-      </c>
-      <c r="I691" s="63">
+      <c r="G691" s="61">
+        <v>60215</v>
+      </c>
+      <c r="H691" s="61">
+        <v>975290</v>
+      </c>
+      <c r="I691" s="61">
         <v>550540</v>
       </c>
-      <c r="J691" s="63">
-        <v>43631</v>
-      </c>
-      <c r="K691" s="63">
-        <v>594171</v>
-      </c>
-      <c r="L691" s="63">
+      <c r="J691" s="61">
+        <v>43702</v>
+      </c>
+      <c r="K691" s="61">
+        <v>594242</v>
+      </c>
+      <c r="L691" s="61">
         <v>1465615</v>
       </c>
-      <c r="M691" s="63">
-        <v>103536</v>
-      </c>
-      <c r="N691" s="63">
-        <v>1569151</v>
-      </c>
-      <c r="O691" s="63">
-        <v>911715</v>
-      </c>
-      <c r="P691" s="63">
+      <c r="M691" s="61">
+        <v>103917</v>
+      </c>
+      <c r="N691" s="61">
+        <v>1569532</v>
+      </c>
+      <c r="O691" s="61">
+        <v>912025</v>
+      </c>
+      <c r="P691" s="61">
         <v>58498</v>
       </c>
-      <c r="Q691" s="63">
+      <c r="Q691" s="61">
         <v>4689</v>
       </c>
       <c r="R691" s="6">
         <v>78</v>
       </c>
-      <c r="S691" s="63">
-        <v>974980</v>
-      </c>
-      <c r="T691" s="63">
-        <v>530354</v>
-      </c>
-      <c r="U691" s="63">
+      <c r="S691" s="61">
+        <v>975290</v>
+      </c>
+      <c r="T691" s="61">
+        <v>530425</v>
+      </c>
+      <c r="U691" s="61">
         <v>60129</v>
       </c>
-      <c r="V691" s="63">
+      <c r="V691" s="61">
         <v>3580</v>
       </c>
       <c r="W691" s="6">
         <v>108</v>
       </c>
-      <c r="X691" s="63">
-        <v>594171</v>
-      </c>
-      <c r="Y691" s="63">
-        <v>1569151</v>
+      <c r="X691" s="61">
+        <v>594242</v>
+      </c>
+      <c r="Y691" s="61">
+        <v>1569532</v>
       </c>
     </row>
     <row r="692" spans="1:25" x14ac:dyDescent="0.25">
@@ -57191,64 +57206,64 @@
       <c r="E692" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F692" s="63">
+      <c r="F692" s="61">
         <v>937765</v>
       </c>
-      <c r="G692" s="63">
+      <c r="G692" s="61">
         <v>12002</v>
       </c>
-      <c r="H692" s="63">
+      <c r="H692" s="61">
         <v>949767</v>
       </c>
-      <c r="I692" s="63">
+      <c r="I692" s="61">
         <v>445313</v>
       </c>
-      <c r="J692" s="63">
+      <c r="J692" s="61">
         <v>15530</v>
       </c>
-      <c r="K692" s="63">
+      <c r="K692" s="61">
         <v>460843</v>
       </c>
-      <c r="L692" s="63">
+      <c r="L692" s="61">
         <v>1383078</v>
       </c>
-      <c r="M692" s="63">
+      <c r="M692" s="61">
         <v>27532</v>
       </c>
-      <c r="N692" s="63">
+      <c r="N692" s="61">
         <v>1410610</v>
       </c>
-      <c r="O692" s="63">
+      <c r="O692" s="61">
         <v>885551</v>
       </c>
-      <c r="P692" s="63">
+      <c r="P692" s="61">
         <v>61516</v>
       </c>
-      <c r="Q692" s="63">
+      <c r="Q692" s="61">
         <v>2678</v>
       </c>
       <c r="R692" s="6">
         <v>22</v>
       </c>
-      <c r="S692" s="63">
+      <c r="S692" s="61">
         <v>949767</v>
       </c>
-      <c r="T692" s="63">
+      <c r="T692" s="61">
         <v>405593</v>
       </c>
-      <c r="U692" s="63">
+      <c r="U692" s="61">
         <v>52483</v>
       </c>
-      <c r="V692" s="63">
+      <c r="V692" s="61">
         <v>2697</v>
       </c>
       <c r="W692" s="6">
         <v>70</v>
       </c>
-      <c r="X692" s="63">
+      <c r="X692" s="61">
         <v>460843</v>
       </c>
-      <c r="Y692" s="63">
+      <c r="Y692" s="61">
         <v>1410610</v>
       </c>
     </row>
@@ -57268,65 +57283,65 @@
       <c r="E693" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F693" s="63">
+      <c r="F693" s="61">
         <v>800679</v>
       </c>
-      <c r="G693" s="63">
-        <v>51711</v>
-      </c>
-      <c r="H693" s="63">
-        <v>852390</v>
-      </c>
-      <c r="I693" s="63">
+      <c r="G693" s="61">
+        <v>51695</v>
+      </c>
+      <c r="H693" s="61">
+        <v>852374</v>
+      </c>
+      <c r="I693" s="61">
         <v>343793</v>
       </c>
-      <c r="J693" s="63">
-        <v>75766</v>
-      </c>
-      <c r="K693" s="63">
-        <v>419559</v>
-      </c>
-      <c r="L693" s="63">
+      <c r="J693" s="61">
+        <v>75694</v>
+      </c>
+      <c r="K693" s="61">
+        <v>419487</v>
+      </c>
+      <c r="L693" s="61">
         <v>1144472</v>
       </c>
-      <c r="M693" s="63">
-        <v>127477</v>
-      </c>
-      <c r="N693" s="63">
-        <v>1271949</v>
-      </c>
-      <c r="O693" s="63">
-        <v>786453</v>
-      </c>
-      <c r="P693" s="63">
+      <c r="M693" s="61">
+        <v>127389</v>
+      </c>
+      <c r="N693" s="61">
+        <v>1271861</v>
+      </c>
+      <c r="O693" s="61">
+        <v>786437</v>
+      </c>
+      <c r="P693" s="61">
         <v>62303</v>
       </c>
-      <c r="Q693" s="63">
+      <c r="Q693" s="61">
         <v>3628</v>
       </c>
       <c r="R693" s="6">
         <v>6</v>
       </c>
-      <c r="S693" s="63">
-        <v>852390</v>
-      </c>
-      <c r="T693" s="63">
-        <v>377966</v>
-      </c>
-      <c r="U693" s="63">
+      <c r="S693" s="61">
+        <v>852374</v>
+      </c>
+      <c r="T693" s="61">
+        <v>377963</v>
+      </c>
+      <c r="U693" s="61">
         <v>40682</v>
       </c>
       <c r="V693" s="6">
-        <v>887</v>
+        <v>818</v>
       </c>
       <c r="W693" s="6">
         <v>24</v>
       </c>
-      <c r="X693" s="63">
-        <v>419559</v>
-      </c>
-      <c r="Y693" s="63">
-        <v>1271949</v>
+      <c r="X693" s="61">
+        <v>419487</v>
+      </c>
+      <c r="Y693" s="61">
+        <v>1271861</v>
       </c>
     </row>
     <row r="694" spans="1:25" x14ac:dyDescent="0.25">
@@ -57345,53 +57360,53 @@
       <c r="E694" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F694" s="63">
+      <c r="F694" s="61">
         <v>637394</v>
       </c>
-      <c r="G694" s="63">
-        <v>1169</v>
-      </c>
-      <c r="H694" s="63">
-        <v>638563</v>
-      </c>
-      <c r="I694" s="63">
+      <c r="G694" s="61">
+        <v>44866</v>
+      </c>
+      <c r="H694" s="61">
+        <v>682260</v>
+      </c>
+      <c r="I694" s="61">
         <v>257890</v>
       </c>
-      <c r="J694" s="63">
-        <v>1542</v>
-      </c>
-      <c r="K694" s="63">
-        <v>259432</v>
-      </c>
-      <c r="L694" s="63">
+      <c r="J694" s="61">
+        <v>3012</v>
+      </c>
+      <c r="K694" s="61">
+        <v>260902</v>
+      </c>
+      <c r="L694" s="61">
         <v>895284</v>
       </c>
-      <c r="M694" s="63">
-        <v>2711</v>
-      </c>
-      <c r="N694" s="63">
-        <v>897995</v>
-      </c>
-      <c r="O694" s="63">
-        <v>573835</v>
-      </c>
-      <c r="P694" s="63">
-        <v>61784</v>
-      </c>
-      <c r="Q694" s="63">
-        <v>2918</v>
+      <c r="M694" s="61">
+        <v>47878</v>
+      </c>
+      <c r="N694" s="61">
+        <v>943162</v>
+      </c>
+      <c r="O694" s="61">
+        <v>615624</v>
+      </c>
+      <c r="P694" s="61">
+        <v>63661</v>
+      </c>
+      <c r="Q694" s="61">
+        <v>2944</v>
       </c>
       <c r="R694" s="6">
-        <v>26</v>
-      </c>
-      <c r="S694" s="63">
-        <v>638563</v>
-      </c>
-      <c r="T694" s="63">
-        <v>230287</v>
-      </c>
-      <c r="U694" s="63">
-        <v>28327</v>
+        <v>31</v>
+      </c>
+      <c r="S694" s="61">
+        <v>682260</v>
+      </c>
+      <c r="T694" s="61">
+        <v>231763</v>
+      </c>
+      <c r="U694" s="61">
+        <v>28321</v>
       </c>
       <c r="V694" s="6">
         <v>783</v>
@@ -57399,11 +57414,11 @@
       <c r="W694" s="6">
         <v>35</v>
       </c>
-      <c r="X694" s="63">
-        <v>259432</v>
-      </c>
-      <c r="Y694" s="63">
-        <v>897995</v>
+      <c r="X694" s="61">
+        <v>260902</v>
+      </c>
+      <c r="Y694" s="61">
+        <v>943162</v>
       </c>
     </row>
     <row r="695" spans="1:25" x14ac:dyDescent="0.25">
@@ -57422,53 +57437,53 @@
       <c r="E695" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F695" s="63">
+      <c r="F695" s="61">
         <v>268544</v>
       </c>
       <c r="G695" s="6">
-        <v>991</v>
-      </c>
-      <c r="H695" s="63">
-        <v>269535</v>
-      </c>
-      <c r="I695" s="63">
+        <v>1029</v>
+      </c>
+      <c r="H695" s="61">
+        <v>269573</v>
+      </c>
+      <c r="I695" s="61">
         <v>85485</v>
       </c>
-      <c r="J695" s="63">
-        <v>2628</v>
-      </c>
-      <c r="K695" s="63">
-        <v>88113</v>
-      </c>
-      <c r="L695" s="63">
+      <c r="J695" s="61">
+        <v>2084</v>
+      </c>
+      <c r="K695" s="61">
+        <v>87569</v>
+      </c>
+      <c r="L695" s="61">
         <v>354029</v>
       </c>
-      <c r="M695" s="63">
-        <v>3619</v>
-      </c>
-      <c r="N695" s="63">
-        <v>357648</v>
-      </c>
-      <c r="O695" s="63">
-        <v>237522</v>
-      </c>
-      <c r="P695" s="63">
+      <c r="M695" s="61">
+        <v>3113</v>
+      </c>
+      <c r="N695" s="61">
+        <v>357142</v>
+      </c>
+      <c r="O695" s="61">
+        <v>237558</v>
+      </c>
+      <c r="P695" s="61">
         <v>30086</v>
       </c>
-      <c r="Q695" s="63">
+      <c r="Q695" s="61">
         <v>1923</v>
       </c>
       <c r="R695" s="6">
-        <v>4</v>
-      </c>
-      <c r="S695" s="63">
-        <v>269535</v>
-      </c>
-      <c r="T695" s="63">
-        <v>80880</v>
-      </c>
-      <c r="U695" s="63">
-        <v>6843</v>
+        <v>6</v>
+      </c>
+      <c r="S695" s="61">
+        <v>269573</v>
+      </c>
+      <c r="T695" s="61">
+        <v>80362</v>
+      </c>
+      <c r="U695" s="61">
+        <v>6817</v>
       </c>
       <c r="V695" s="6">
         <v>86</v>
@@ -57476,11 +57491,11 @@
       <c r="W695" s="6">
         <v>304</v>
       </c>
-      <c r="X695" s="63">
-        <v>88113</v>
-      </c>
-      <c r="Y695" s="63">
-        <v>357648</v>
+      <c r="X695" s="61">
+        <v>87569</v>
+      </c>
+      <c r="Y695" s="61">
+        <v>357142</v>
       </c>
     </row>
     <row r="696" spans="1:25" x14ac:dyDescent="0.25">
@@ -57499,52 +57514,52 @@
       <c r="E696" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F696" s="63">
+      <c r="F696" s="61">
         <v>432804</v>
       </c>
-      <c r="G696" s="63">
-        <v>-5334</v>
-      </c>
-      <c r="H696" s="63">
-        <v>427470</v>
-      </c>
-      <c r="I696" s="63">
+      <c r="G696" s="61">
+        <v>-8477</v>
+      </c>
+      <c r="H696" s="61">
+        <v>424327</v>
+      </c>
+      <c r="I696" s="61">
         <v>150038</v>
       </c>
       <c r="J696" s="6">
-        <v>956</v>
-      </c>
-      <c r="K696" s="63">
-        <v>150994</v>
-      </c>
-      <c r="L696" s="63">
+        <v>-63</v>
+      </c>
+      <c r="K696" s="61">
+        <v>149975</v>
+      </c>
+      <c r="L696" s="61">
         <v>582842</v>
       </c>
-      <c r="M696" s="63">
-        <v>-4378</v>
-      </c>
-      <c r="N696" s="63">
-        <v>578464</v>
-      </c>
-      <c r="O696" s="63">
-        <v>374492</v>
-      </c>
-      <c r="P696" s="63">
-        <v>48627</v>
-      </c>
-      <c r="Q696" s="63">
+      <c r="M696" s="61">
+        <v>-8540</v>
+      </c>
+      <c r="N696" s="61">
+        <v>574302</v>
+      </c>
+      <c r="O696" s="61">
+        <v>372736</v>
+      </c>
+      <c r="P696" s="61">
+        <v>47240</v>
+      </c>
+      <c r="Q696" s="61">
         <v>4323</v>
       </c>
       <c r="R696" s="6">
         <v>28</v>
       </c>
-      <c r="S696" s="63">
-        <v>427470</v>
-      </c>
-      <c r="T696" s="63">
-        <v>135106</v>
-      </c>
-      <c r="U696" s="63">
+      <c r="S696" s="61">
+        <v>424327</v>
+      </c>
+      <c r="T696" s="61">
+        <v>134087</v>
+      </c>
+      <c r="U696" s="61">
         <v>15007</v>
       </c>
       <c r="V696" s="6">
@@ -57553,11 +57568,11 @@
       <c r="W696" s="6">
         <v>7</v>
       </c>
-      <c r="X696" s="63">
-        <v>150994</v>
-      </c>
-      <c r="Y696" s="63">
-        <v>578464</v>
+      <c r="X696" s="61">
+        <v>149975</v>
+      </c>
+      <c r="Y696" s="61">
+        <v>574302</v>
       </c>
     </row>
     <row r="697" spans="1:25" x14ac:dyDescent="0.25">
@@ -57567,7 +57582,7 @@
       <c r="B697" s="4">
         <v>26</v>
       </c>
-      <c r="C697" s="60" t="s">
+      <c r="C697" s="59" t="s">
         <v>738</v>
       </c>
       <c r="D697" s="6" t="s">
@@ -57576,53 +57591,53 @@
       <c r="E697" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F697" s="63">
+      <c r="F697" s="61">
         <v>260568</v>
       </c>
-      <c r="G697" s="63">
-        <v>4183</v>
-      </c>
-      <c r="H697" s="63">
-        <v>264751</v>
-      </c>
-      <c r="I697" s="63">
+      <c r="G697" s="61">
+        <v>23532</v>
+      </c>
+      <c r="H697" s="61">
+        <v>284100</v>
+      </c>
+      <c r="I697" s="61">
         <v>109681</v>
       </c>
-      <c r="J697" s="63">
-        <v>8812</v>
-      </c>
-      <c r="K697" s="63">
-        <v>118493</v>
-      </c>
-      <c r="L697" s="63">
+      <c r="J697" s="61">
+        <v>42586</v>
+      </c>
+      <c r="K697" s="61">
+        <v>152267</v>
+      </c>
+      <c r="L697" s="61">
         <v>370249</v>
       </c>
-      <c r="M697" s="63">
-        <v>12995</v>
-      </c>
-      <c r="N697" s="63">
-        <v>383244</v>
-      </c>
-      <c r="O697" s="63">
-        <v>234920</v>
-      </c>
-      <c r="P697" s="63">
+      <c r="M697" s="61">
+        <v>66118</v>
+      </c>
+      <c r="N697" s="61">
+        <v>436367</v>
+      </c>
+      <c r="O697" s="61">
+        <v>254269</v>
+      </c>
+      <c r="P697" s="61">
         <v>26757</v>
       </c>
-      <c r="Q697" s="63">
+      <c r="Q697" s="61">
         <v>3065</v>
       </c>
       <c r="R697" s="6">
         <v>9</v>
       </c>
-      <c r="S697" s="63">
-        <v>264751</v>
-      </c>
-      <c r="T697" s="63">
-        <v>109955</v>
-      </c>
-      <c r="U697" s="63">
-        <v>8174</v>
+      <c r="S697" s="61">
+        <v>284100</v>
+      </c>
+      <c r="T697" s="61">
+        <v>143762</v>
+      </c>
+      <c r="U697" s="61">
+        <v>8141</v>
       </c>
       <c r="V697" s="6">
         <v>304</v>
@@ -57630,11 +57645,11 @@
       <c r="W697" s="6">
         <v>60</v>
       </c>
-      <c r="X697" s="63">
-        <v>118493</v>
-      </c>
-      <c r="Y697" s="63">
-        <v>383244</v>
+      <c r="X697" s="61">
+        <v>152267</v>
+      </c>
+      <c r="Y697" s="61">
+        <v>436367</v>
       </c>
     </row>
     <row r="698" spans="1:25" x14ac:dyDescent="0.25">
@@ -57644,7 +57659,7 @@
       <c r="B698" s="4">
         <v>27</v>
       </c>
-      <c r="C698" s="60" t="s">
+      <c r="C698" s="59" t="s">
         <v>739</v>
       </c>
       <c r="D698" s="6" t="s">
@@ -57653,53 +57668,53 @@
       <c r="E698" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F698" s="63">
+      <c r="F698" s="61">
         <v>146617</v>
       </c>
       <c r="G698" s="6">
-        <v>0</v>
-      </c>
-      <c r="H698" s="63">
-        <v>146617</v>
-      </c>
-      <c r="I698" s="63">
+        <v>1627</v>
+      </c>
+      <c r="H698" s="61">
+        <v>148244</v>
+      </c>
+      <c r="I698" s="61">
         <v>77228</v>
       </c>
       <c r="J698" s="6">
-        <v>0</v>
-      </c>
-      <c r="K698" s="63">
-        <v>77228</v>
-      </c>
-      <c r="L698" s="63">
+        <v>1687</v>
+      </c>
+      <c r="K698" s="61">
+        <v>78915</v>
+      </c>
+      <c r="L698" s="61">
         <v>223845</v>
       </c>
       <c r="M698" s="6">
-        <v>0</v>
-      </c>
-      <c r="N698" s="63">
-        <v>223845</v>
-      </c>
-      <c r="O698" s="63">
-        <v>130250</v>
-      </c>
-      <c r="P698" s="63">
-        <v>14724</v>
-      </c>
-      <c r="Q698" s="63">
-        <v>1588</v>
+        <v>3314</v>
+      </c>
+      <c r="N698" s="61">
+        <v>227159</v>
+      </c>
+      <c r="O698" s="61">
+        <v>131622</v>
+      </c>
+      <c r="P698" s="61">
+        <v>14941</v>
+      </c>
+      <c r="Q698" s="61">
+        <v>1626</v>
       </c>
       <c r="R698" s="6">
         <v>55</v>
       </c>
-      <c r="S698" s="63">
-        <v>146617</v>
-      </c>
-      <c r="T698" s="63">
-        <v>71292</v>
-      </c>
-      <c r="U698" s="63">
-        <v>5916</v>
+      <c r="S698" s="61">
+        <v>148244</v>
+      </c>
+      <c r="T698" s="61">
+        <v>72676</v>
+      </c>
+      <c r="U698" s="61">
+        <v>6219</v>
       </c>
       <c r="V698" s="6">
         <v>20</v>
@@ -57707,11 +57722,11 @@
       <c r="W698" s="6">
         <v>0</v>
       </c>
-      <c r="X698" s="63">
-        <v>77228</v>
-      </c>
-      <c r="Y698" s="63">
-        <v>223845</v>
+      <c r="X698" s="61">
+        <v>78915</v>
+      </c>
+      <c r="Y698" s="61">
+        <v>227159</v>
       </c>
     </row>
     <row r="699" spans="1:25" x14ac:dyDescent="0.25">
@@ -57721,33 +57736,75 @@
       <c r="B699" s="4">
         <v>28</v>
       </c>
-      <c r="C699" s="7"/>
+      <c r="C699" s="59" t="s">
+        <v>740</v>
+      </c>
       <c r="D699" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E699" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F699" s="6"/>
-      <c r="G699" s="6"/>
-      <c r="H699" s="6"/>
-      <c r="I699" s="6"/>
-      <c r="J699" s="6"/>
-      <c r="K699" s="6"/>
-      <c r="L699" s="6"/>
-      <c r="M699" s="6"/>
-      <c r="N699" s="6"/>
-      <c r="O699" s="6"/>
-      <c r="P699" s="6"/>
-      <c r="Q699" s="6"/>
-      <c r="R699" s="6"/>
-      <c r="S699" s="6"/>
-      <c r="T699" s="6"/>
-      <c r="U699" s="6"/>
-      <c r="V699" s="6"/>
-      <c r="W699" s="6"/>
-      <c r="X699" s="6"/>
-      <c r="Y699" s="6"/>
+      <c r="F699" s="6">
+        <v>64631</v>
+      </c>
+      <c r="G699" s="6">
+        <v>50</v>
+      </c>
+      <c r="H699" s="6">
+        <v>64681</v>
+      </c>
+      <c r="I699" s="6">
+        <v>43602</v>
+      </c>
+      <c r="J699" s="6">
+        <v>545</v>
+      </c>
+      <c r="K699" s="6">
+        <v>44147</v>
+      </c>
+      <c r="L699" s="6">
+        <v>108233</v>
+      </c>
+      <c r="M699" s="6">
+        <v>595</v>
+      </c>
+      <c r="N699" s="6">
+        <v>108828</v>
+      </c>
+      <c r="O699" s="6">
+        <v>57469</v>
+      </c>
+      <c r="P699" s="6">
+        <v>6144</v>
+      </c>
+      <c r="Q699" s="6">
+        <v>1020</v>
+      </c>
+      <c r="R699" s="6">
+        <v>48</v>
+      </c>
+      <c r="S699" s="6">
+        <v>64681</v>
+      </c>
+      <c r="T699" s="6">
+        <v>42770</v>
+      </c>
+      <c r="U699" s="6">
+        <v>1225</v>
+      </c>
+      <c r="V699" s="6">
+        <v>149</v>
+      </c>
+      <c r="W699" s="6">
+        <v>3</v>
+      </c>
+      <c r="X699" s="6">
+        <v>44147</v>
+      </c>
+      <c r="Y699" s="6">
+        <v>108828</v>
+      </c>
     </row>
     <row r="700" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A700" s="7">
@@ -57756,33 +57813,75 @@
       <c r="B700" s="4">
         <v>29</v>
       </c>
-      <c r="C700" s="7"/>
+      <c r="C700" s="59" t="s">
+        <v>741</v>
+      </c>
       <c r="D700" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E700" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F700" s="6"/>
-      <c r="G700" s="6"/>
-      <c r="H700" s="6"/>
-      <c r="I700" s="6"/>
-      <c r="J700" s="6"/>
-      <c r="K700" s="6"/>
-      <c r="L700" s="6"/>
-      <c r="M700" s="6"/>
-      <c r="N700" s="6"/>
-      <c r="O700" s="6"/>
-      <c r="P700" s="6"/>
-      <c r="Q700" s="6"/>
-      <c r="R700" s="6"/>
-      <c r="S700" s="6"/>
-      <c r="T700" s="6"/>
-      <c r="U700" s="6"/>
-      <c r="V700" s="6"/>
-      <c r="W700" s="6"/>
-      <c r="X700" s="6"/>
-      <c r="Y700" s="6"/>
+      <c r="F700" s="6">
+        <v>70979</v>
+      </c>
+      <c r="G700" s="6">
+        <v>1159</v>
+      </c>
+      <c r="H700" s="6">
+        <v>72138</v>
+      </c>
+      <c r="I700" s="6">
+        <v>37825</v>
+      </c>
+      <c r="J700" s="6">
+        <v>1725</v>
+      </c>
+      <c r="K700" s="6">
+        <v>39550</v>
+      </c>
+      <c r="L700" s="6">
+        <v>108804</v>
+      </c>
+      <c r="M700" s="6">
+        <v>2884</v>
+      </c>
+      <c r="N700" s="6">
+        <v>111688</v>
+      </c>
+      <c r="O700" s="6">
+        <v>65210</v>
+      </c>
+      <c r="P700" s="6">
+        <v>6336</v>
+      </c>
+      <c r="Q700" s="6">
+        <v>547</v>
+      </c>
+      <c r="R700" s="6">
+        <v>45</v>
+      </c>
+      <c r="S700" s="6">
+        <v>72138</v>
+      </c>
+      <c r="T700" s="6">
+        <v>38468</v>
+      </c>
+      <c r="U700" s="6">
+        <v>887</v>
+      </c>
+      <c r="V700" s="6">
+        <v>195</v>
+      </c>
+      <c r="W700" s="6">
+        <v>0</v>
+      </c>
+      <c r="X700" s="6">
+        <v>39550</v>
+      </c>
+      <c r="Y700" s="6">
+        <v>111688</v>
+      </c>
     </row>
     <row r="701" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A701" s="7">
@@ -57791,33 +57890,75 @@
       <c r="B701" s="4">
         <v>30</v>
       </c>
-      <c r="C701" s="7"/>
+      <c r="C701" s="59" t="s">
+        <v>742</v>
+      </c>
       <c r="D701" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E701" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F701" s="6"/>
-      <c r="G701" s="6"/>
-      <c r="H701" s="6"/>
-      <c r="I701" s="6"/>
-      <c r="J701" s="6"/>
-      <c r="K701" s="6"/>
-      <c r="L701" s="6"/>
-      <c r="M701" s="6"/>
-      <c r="N701" s="6"/>
-      <c r="O701" s="6"/>
-      <c r="P701" s="6"/>
-      <c r="Q701" s="6"/>
-      <c r="R701" s="6"/>
-      <c r="S701" s="6"/>
-      <c r="T701" s="6"/>
-      <c r="U701" s="6"/>
-      <c r="V701" s="6"/>
-      <c r="W701" s="6"/>
-      <c r="X701" s="6"/>
-      <c r="Y701" s="6"/>
+      <c r="F701" s="6">
+        <v>49909</v>
+      </c>
+      <c r="G701" s="6">
+        <v>7974</v>
+      </c>
+      <c r="H701" s="6">
+        <v>57883</v>
+      </c>
+      <c r="I701" s="6">
+        <v>30670</v>
+      </c>
+      <c r="J701" s="6">
+        <v>7058</v>
+      </c>
+      <c r="K701" s="6">
+        <v>37728</v>
+      </c>
+      <c r="L701" s="6">
+        <v>80579</v>
+      </c>
+      <c r="M701" s="6">
+        <v>15032</v>
+      </c>
+      <c r="N701" s="6">
+        <v>95611</v>
+      </c>
+      <c r="O701" s="6">
+        <v>52748</v>
+      </c>
+      <c r="P701" s="6">
+        <v>4563</v>
+      </c>
+      <c r="Q701" s="6">
+        <v>544</v>
+      </c>
+      <c r="R701" s="6">
+        <v>28</v>
+      </c>
+      <c r="S701" s="6">
+        <v>57883</v>
+      </c>
+      <c r="T701" s="6">
+        <v>36962</v>
+      </c>
+      <c r="U701" s="6">
+        <v>651</v>
+      </c>
+      <c r="V701" s="6">
+        <v>115</v>
+      </c>
+      <c r="W701" s="6">
+        <v>0</v>
+      </c>
+      <c r="X701" s="6">
+        <v>37728</v>
+      </c>
+      <c r="Y701" s="6">
+        <v>95611</v>
+      </c>
     </row>
     <row r="702" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A702" s="7">
@@ -57826,33 +57967,75 @@
       <c r="B702" s="4">
         <v>31</v>
       </c>
-      <c r="C702" s="7"/>
+      <c r="C702" s="59" t="s">
+        <v>743</v>
+      </c>
       <c r="D702" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E702" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F702" s="6"/>
-      <c r="G702" s="6"/>
-      <c r="H702" s="6"/>
-      <c r="I702" s="6"/>
-      <c r="J702" s="6"/>
-      <c r="K702" s="6"/>
-      <c r="L702" s="6"/>
-      <c r="M702" s="6"/>
-      <c r="N702" s="6"/>
-      <c r="O702" s="6"/>
-      <c r="P702" s="6"/>
-      <c r="Q702" s="6"/>
-      <c r="R702" s="6"/>
-      <c r="S702" s="6"/>
-      <c r="T702" s="6"/>
-      <c r="U702" s="6"/>
-      <c r="V702" s="6"/>
-      <c r="W702" s="6"/>
-      <c r="X702" s="6"/>
-      <c r="Y702" s="6"/>
+      <c r="F702" s="6">
+        <v>38426</v>
+      </c>
+      <c r="G702" s="6">
+        <v>-355</v>
+      </c>
+      <c r="H702" s="6">
+        <v>38071</v>
+      </c>
+      <c r="I702" s="6">
+        <v>31328</v>
+      </c>
+      <c r="J702" s="6">
+        <v>659</v>
+      </c>
+      <c r="K702" s="6">
+        <v>31987</v>
+      </c>
+      <c r="L702" s="6">
+        <v>69754</v>
+      </c>
+      <c r="M702" s="6">
+        <v>304</v>
+      </c>
+      <c r="N702" s="6">
+        <v>70058</v>
+      </c>
+      <c r="O702" s="6">
+        <v>34766</v>
+      </c>
+      <c r="P702" s="6">
+        <v>2498</v>
+      </c>
+      <c r="Q702" s="6">
+        <v>790</v>
+      </c>
+      <c r="R702" s="6">
+        <v>17</v>
+      </c>
+      <c r="S702" s="6">
+        <v>38071</v>
+      </c>
+      <c r="T702" s="6">
+        <v>31226</v>
+      </c>
+      <c r="U702" s="6">
+        <v>533</v>
+      </c>
+      <c r="V702" s="6">
+        <v>228</v>
+      </c>
+      <c r="W702" s="6">
+        <v>0</v>
+      </c>
+      <c r="X702" s="6">
+        <v>31987</v>
+      </c>
+      <c r="Y702" s="6">
+        <v>70058</v>
+      </c>
     </row>
     <row r="703" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A703" s="7">
@@ -57861,33 +58044,75 @@
       <c r="B703" s="4">
         <v>32</v>
       </c>
-      <c r="C703" s="7"/>
+      <c r="C703" s="60" t="s">
+        <v>744</v>
+      </c>
       <c r="D703" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E703" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F703" s="6"/>
-      <c r="G703" s="6"/>
-      <c r="H703" s="6"/>
-      <c r="I703" s="6"/>
-      <c r="J703" s="6"/>
-      <c r="K703" s="6"/>
-      <c r="L703" s="6"/>
-      <c r="M703" s="6"/>
-      <c r="N703" s="6"/>
-      <c r="O703" s="6"/>
-      <c r="P703" s="6"/>
-      <c r="Q703" s="6"/>
-      <c r="R703" s="6"/>
-      <c r="S703" s="6"/>
-      <c r="T703" s="6"/>
-      <c r="U703" s="6"/>
-      <c r="V703" s="6"/>
-      <c r="W703" s="6"/>
-      <c r="X703" s="6"/>
-      <c r="Y703" s="6"/>
+      <c r="F703" s="6">
+        <v>57346</v>
+      </c>
+      <c r="G703" s="6">
+        <v>0</v>
+      </c>
+      <c r="H703" s="6">
+        <v>57346</v>
+      </c>
+      <c r="I703" s="6">
+        <v>27984</v>
+      </c>
+      <c r="J703" s="6">
+        <v>0</v>
+      </c>
+      <c r="K703" s="6">
+        <v>27984</v>
+      </c>
+      <c r="L703" s="6">
+        <v>85330</v>
+      </c>
+      <c r="M703" s="6">
+        <v>0</v>
+      </c>
+      <c r="N703" s="6">
+        <v>85330</v>
+      </c>
+      <c r="O703" s="6">
+        <v>53420</v>
+      </c>
+      <c r="P703" s="6">
+        <v>2967</v>
+      </c>
+      <c r="Q703" s="6">
+        <v>922</v>
+      </c>
+      <c r="R703" s="6">
+        <v>37</v>
+      </c>
+      <c r="S703" s="6">
+        <v>57346</v>
+      </c>
+      <c r="T703" s="6">
+        <v>27652</v>
+      </c>
+      <c r="U703" s="6">
+        <v>219</v>
+      </c>
+      <c r="V703" s="6">
+        <v>113</v>
+      </c>
+      <c r="W703" s="6">
+        <v>0</v>
+      </c>
+      <c r="X703" s="6">
+        <v>27984</v>
+      </c>
+      <c r="Y703" s="6">
+        <v>85330</v>
+      </c>
     </row>
     <row r="704" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A704" s="7">
@@ -58859,17 +59084,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075ECE796D7EABA42BC0DB2CA73C7CE00" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e2ecee1b3d34a959aed38d5dc4c878f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8" xmlns:ns3="ae149517-eeaa-465d-b3b6-396a1e23bc6e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9af26d9f7c79c0f2a842447557dfee25" ns2:_="" ns3:_="">
     <xsd:import namespace="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
@@ -59096,6 +59310,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -59106,17 +59331,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
-    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A42C790-3343-4FC1-9ABA-46A7C5CDBF94}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -59135,6 +59349,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
+    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
   <ds:schemaRefs>

</xml_diff>